<commit_message>
Improves metadata assets incremental build performance.
</commit_message>
<xml_diff>
--- a/SampleExcelFiles/GenericTypeSampleMetadata.xlsx
+++ b/SampleExcelFiles/GenericTypeSampleMetadata.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/External/Projects/GitHub/UniSharper.Data.Metadata/master/SampleExcelFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B0F479A-0BC2-E649-9ECF-9DAF62F34A0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D62A3970-34EA-5248-9C92-2060B93A7211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1480" yWindow="1660" windowWidth="38400" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="104">
   <si>
     <t>long</t>
   </si>
@@ -433,6 +433,10 @@
   </si>
   <si>
     <t>dsaweq你好！@#￥%……&amp;*（）</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1227,8 +1231,8 @@
       <c r="I4" s="5">
         <v>2147483647</v>
       </c>
-      <c r="J4" s="5">
-        <v>0</v>
+      <c r="J4" s="5" t="s">
+        <v>103</v>
       </c>
       <c r="K4" s="6">
         <v>-922337203685477</v>

</xml_diff>

<commit_message>
Changed the method for retrieving the modified time of .xlsx files.
</commit_message>
<xml_diff>
--- a/SampleExcelFiles/GenericTypeSampleMetadata.xlsx
+++ b/SampleExcelFiles/GenericTypeSampleMetadata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/External/Projects/GitHub/UniSharper.Data.Metadata/master/SampleExcelFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D62A3970-34EA-5248-9C92-2060B93A7211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF6084B4-52A2-F548-93BE-BB50F9BFCDC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1480" yWindow="1660" windowWidth="38400" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="105">
   <si>
     <t>long</t>
   </si>
@@ -437,6 +437,10 @@
   </si>
   <si>
     <t>1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1225,8 +1229,8 @@
       <c r="G4" s="5">
         <v>-32768</v>
       </c>
-      <c r="H4" s="5">
-        <v>0</v>
+      <c r="H4" s="5" t="s">
+        <v>104</v>
       </c>
       <c r="I4" s="5">
         <v>2147483647</v>

</xml_diff>